<commit_message>
fix: graphics not showing in EDA page
</commit_message>
<xml_diff>
--- a/uploads/dataset/output/bab4/summary_statistic.xlsx
+++ b/uploads/dataset/output/bab4/summary_statistic.xlsx
@@ -496,7 +496,7 @@
         <v>2531</v>
       </c>
       <c r="D2" t="n">
-        <v>2530</v>
+        <v>2531</v>
       </c>
       <c r="E2" t="n">
         <v>2531</v>
@@ -523,7 +523,7 @@
         <v>2531</v>
       </c>
       <c r="M2" t="n">
-        <v>2530</v>
+        <v>2531</v>
       </c>
       <c r="N2" t="n">
         <v>2531</v>
@@ -542,7 +542,7 @@
         <v>604.4207822994864</v>
       </c>
       <c r="D3" t="n">
-        <v>7.756251857707509</v>
+        <v>7.756217779533781</v>
       </c>
       <c r="E3" t="n">
         <v>129.1592256025286</v>
@@ -569,7 +569,7 @@
         <v>74.35784315016164</v>
       </c>
       <c r="M3" t="n">
-        <v>-0.04660047430830039</v>
+        <v>-0.0465227973133149</v>
       </c>
       <c r="N3" t="n">
         <v>1322.807172540498</v>
@@ -588,7 +588,7 @@
         <v>291.8912237609017</v>
       </c>
       <c r="D4" t="n">
-        <v>0.2366935300914174</v>
+        <v>0.2366529583329053</v>
       </c>
       <c r="E4" t="n">
         <v>47.73202052534224</v>
@@ -615,7 +615,7 @@
         <v>13.57706593162572</v>
       </c>
       <c r="M4" t="n">
-        <v>0.2563364618086981</v>
+        <v>0.2563155892533779</v>
       </c>
       <c r="N4" t="n">
         <v>884.8918976874141</v>

</xml_diff>